<commit_message>
Sorry, it was 1.16
</commit_message>
<xml_diff>
--- a/SimonCani_glyphs.xlsx
+++ b/SimonCani_glyphs.xlsx
@@ -44,15 +44,7 @@
     <t>GlyphName</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>□</t>
-    </r>
+    <t>□</t>
   </si>
   <si>
     <t>\u0000</t>
@@ -4210,6 +4202,12 @@
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -4354,12 +4352,6 @@
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="33">
@@ -4695,16 +4687,13 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -4713,119 +4702,122 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4835,6 +4827,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -5183,7 +5178,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E352"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" customHeight="1" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="9.25" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.25" customWidth="1"/>
@@ -5192,7 +5187,7 @@
     <col min="5" max="5" width="29.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" customHeight="1" spans="1:5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5209,8 +5204,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="13.5" spans="1:5">
-      <c r="A2" s="1" t="s">
+    <row r="2" customHeight="1" spans="1:5">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
@@ -5226,7 +5221,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" customHeight="1" spans="1:5">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -5243,7 +5238,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" customHeight="1" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -5260,7 +5255,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" customHeight="1" spans="1:5">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -5277,7 +5272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" customHeight="1" spans="1:5">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -5294,7 +5289,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" customHeight="1" spans="1:5">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -5311,7 +5306,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" customHeight="1" spans="1:5">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -5328,7 +5323,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" customHeight="1" spans="1:5">
       <c r="A9" s="1" t="s">
         <v>34</v>
       </c>
@@ -5345,7 +5340,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" customHeight="1" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
@@ -5362,7 +5357,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" customHeight="1" spans="1:5">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -5379,7 +5374,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" customHeight="1" spans="1:5">
       <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
@@ -5396,7 +5391,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" customHeight="1" spans="1:5">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -5413,7 +5408,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" customHeight="1" spans="1:5">
       <c r="A14" s="1" t="s">
         <v>54</v>
       </c>
@@ -5430,7 +5425,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" customHeight="1" spans="1:5">
       <c r="A15" s="1" t="s">
         <v>58</v>
       </c>
@@ -5447,7 +5442,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" customHeight="1" spans="1:5">
       <c r="A16" s="1" t="s">
         <v>62</v>
       </c>
@@ -5464,7 +5459,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" customHeight="1" spans="1:5">
       <c r="A17" s="1" t="s">
         <v>66</v>
       </c>
@@ -5481,7 +5476,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" customHeight="1" spans="1:5">
       <c r="A18" s="1" t="s">
         <v>70</v>
       </c>
@@ -5498,7 +5493,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" customHeight="1" spans="1:5">
       <c r="A19" s="1" t="s">
         <v>74</v>
       </c>
@@ -5515,7 +5510,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" customHeight="1" spans="1:5">
       <c r="A20" s="1" t="s">
         <v>78</v>
       </c>
@@ -5532,7 +5527,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" customHeight="1" spans="1:5">
       <c r="A21" s="1" t="s">
         <v>82</v>
       </c>
@@ -5549,7 +5544,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" customHeight="1" spans="1:5">
       <c r="A22" s="1" t="s">
         <v>86</v>
       </c>
@@ -5566,7 +5561,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" customHeight="1" spans="1:5">
       <c r="A23" s="1" t="s">
         <v>90</v>
       </c>
@@ -5583,7 +5578,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" customHeight="1" spans="1:5">
       <c r="A24" s="1" t="s">
         <v>94</v>
       </c>
@@ -5600,7 +5595,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" customHeight="1" spans="1:5">
       <c r="A25" s="1" t="s">
         <v>98</v>
       </c>
@@ -5617,7 +5612,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" customHeight="1" spans="1:5">
       <c r="A26" s="1" t="s">
         <v>102</v>
       </c>
@@ -5634,7 +5629,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" customHeight="1" spans="1:5">
       <c r="A27" s="1" t="s">
         <v>106</v>
       </c>
@@ -5651,7 +5646,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" customHeight="1" spans="1:5">
       <c r="A28" s="1" t="s">
         <v>110</v>
       </c>
@@ -5668,7 +5663,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" customHeight="1" spans="1:5">
       <c r="A29" s="1" t="s">
         <v>114</v>
       </c>
@@ -5685,7 +5680,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" customHeight="1" spans="1:5">
       <c r="A30" s="1" t="s">
         <v>118</v>
       </c>
@@ -5702,7 +5697,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" customHeight="1" spans="1:5">
       <c r="A31" s="1" t="s">
         <v>122</v>
       </c>
@@ -5719,7 +5714,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" customHeight="1" spans="1:5">
       <c r="A32" s="1" t="s">
         <v>126</v>
       </c>
@@ -5736,7 +5731,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" customHeight="1" spans="1:5">
       <c r="A33" s="1" t="s">
         <v>130</v>
       </c>
@@ -5753,7 +5748,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" customHeight="1" spans="1:5">
       <c r="A34" s="1" t="s">
         <v>134</v>
       </c>
@@ -5770,7 +5765,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" customHeight="1" spans="1:5">
       <c r="A35" s="1" t="s">
         <v>138</v>
       </c>
@@ -5787,7 +5782,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" customHeight="1" spans="1:5">
       <c r="A36" s="1" t="s">
         <v>142</v>
       </c>
@@ -5804,7 +5799,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" customHeight="1" spans="1:5">
       <c r="A37" s="1" t="s">
         <v>146</v>
       </c>
@@ -5821,7 +5816,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" customHeight="1" spans="1:5">
       <c r="A38" s="1" t="s">
         <v>150</v>
       </c>
@@ -5838,7 +5833,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" customHeight="1" spans="1:5">
       <c r="A39" s="1" t="s">
         <v>154</v>
       </c>
@@ -5855,7 +5850,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" customHeight="1" spans="1:5">
       <c r="A40" s="1" t="s">
         <v>158</v>
       </c>
@@ -5872,7 +5867,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" customHeight="1" spans="1:5">
       <c r="A41" s="1" t="s">
         <v>162</v>
       </c>
@@ -5889,7 +5884,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" customHeight="1" spans="1:5">
       <c r="A42" s="1" t="s">
         <v>166</v>
       </c>
@@ -5906,7 +5901,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" customHeight="1" spans="1:5">
       <c r="A43" s="1" t="s">
         <v>170</v>
       </c>
@@ -5923,7 +5918,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" customHeight="1" spans="1:5">
       <c r="A44" s="1" t="s">
         <v>174</v>
       </c>
@@ -5940,7 +5935,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" customHeight="1" spans="1:5">
       <c r="A45" s="1" t="s">
         <v>178</v>
       </c>
@@ -5957,7 +5952,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" customHeight="1" spans="1:5">
       <c r="A46" s="1" t="s">
         <v>182</v>
       </c>
@@ -5974,7 +5969,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" customHeight="1" spans="1:5">
       <c r="A47" s="1" t="s">
         <v>186</v>
       </c>
@@ -5991,7 +5986,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" customHeight="1" spans="1:5">
       <c r="A48" s="1" t="s">
         <v>190</v>
       </c>
@@ -6008,7 +6003,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" customHeight="1" spans="1:5">
       <c r="A49" s="1" t="s">
         <v>194</v>
       </c>
@@ -6025,7 +6020,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" customHeight="1" spans="1:5">
       <c r="A50" s="1" t="s">
         <v>198</v>
       </c>
@@ -6042,7 +6037,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" customHeight="1" spans="1:5">
       <c r="A51" s="1" t="s">
         <v>202</v>
       </c>
@@ -6059,7 +6054,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" customHeight="1" spans="1:5">
       <c r="A52" s="1" t="s">
         <v>206</v>
       </c>
@@ -6076,7 +6071,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" customHeight="1" spans="1:5">
       <c r="A53" s="1" t="s">
         <v>210</v>
       </c>
@@ -6093,7 +6088,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" customHeight="1" spans="1:5">
       <c r="A54" s="1" t="s">
         <v>214</v>
       </c>
@@ -6110,7 +6105,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" customHeight="1" spans="1:5">
       <c r="A55" s="1" t="s">
         <v>218</v>
       </c>
@@ -6127,7 +6122,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" customHeight="1" spans="1:5">
       <c r="A56" s="1" t="s">
         <v>222</v>
       </c>
@@ -6144,7 +6139,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" customHeight="1" spans="1:5">
       <c r="A57" s="1" t="s">
         <v>226</v>
       </c>
@@ -6161,7 +6156,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" customHeight="1" spans="1:5">
       <c r="A58" s="1" t="s">
         <v>230</v>
       </c>
@@ -6178,7 +6173,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" customHeight="1" spans="1:5">
       <c r="A59" s="1" t="s">
         <v>234</v>
       </c>
@@ -6195,7 +6190,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" customHeight="1" spans="1:5">
       <c r="A60" s="1" t="s">
         <v>238</v>
       </c>
@@ -6212,7 +6207,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" customHeight="1" spans="1:5">
       <c r="A61" s="1" t="s">
         <v>242</v>
       </c>
@@ -6229,7 +6224,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" customHeight="1" spans="1:5">
       <c r="A62" s="1" t="s">
         <v>246</v>
       </c>
@@ -6246,7 +6241,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" customHeight="1" spans="1:5">
       <c r="A63" s="1" t="s">
         <v>250</v>
       </c>
@@ -6263,7 +6258,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" customHeight="1" spans="1:5">
       <c r="A64" s="1" t="s">
         <v>254</v>
       </c>
@@ -6280,7 +6275,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" customHeight="1" spans="1:5">
       <c r="A65" s="1" t="s">
         <v>258</v>
       </c>
@@ -6297,7 +6292,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" customHeight="1" spans="1:5">
       <c r="A66" s="1" t="s">
         <v>262</v>
       </c>
@@ -6314,7 +6309,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" customHeight="1" spans="1:5">
       <c r="A67" s="1" t="s">
         <v>266</v>
       </c>
@@ -6331,7 +6326,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" customHeight="1" spans="1:5">
       <c r="A68" s="1" t="s">
         <v>270</v>
       </c>
@@ -6348,7 +6343,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" customHeight="1" spans="1:5">
       <c r="A69" s="1" t="s">
         <v>274</v>
       </c>
@@ -6365,7 +6360,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" customHeight="1" spans="1:5">
       <c r="A70" s="1" t="s">
         <v>278</v>
       </c>
@@ -6382,7 +6377,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" customHeight="1" spans="1:5">
       <c r="A71" s="1" t="s">
         <v>282</v>
       </c>
@@ -6399,7 +6394,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" customHeight="1" spans="1:5">
       <c r="A72" s="1" t="s">
         <v>286</v>
       </c>
@@ -6416,7 +6411,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" customHeight="1" spans="1:5">
       <c r="A73" s="1" t="s">
         <v>290</v>
       </c>
@@ -6433,7 +6428,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" customHeight="1" spans="1:5">
       <c r="A74" s="1" t="s">
         <v>294</v>
       </c>
@@ -6450,7 +6445,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" customHeight="1" spans="1:5">
       <c r="A75" s="1" t="s">
         <v>298</v>
       </c>
@@ -6467,7 +6462,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" customHeight="1" spans="1:5">
       <c r="A76" s="1" t="s">
         <v>302</v>
       </c>
@@ -6484,7 +6479,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" customHeight="1" spans="1:5">
       <c r="A77" s="1" t="s">
         <v>306</v>
       </c>
@@ -6501,7 +6496,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" customHeight="1" spans="1:5">
       <c r="A78" s="1" t="s">
         <v>310</v>
       </c>
@@ -6518,7 +6513,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" customHeight="1" spans="1:5">
       <c r="A79" s="1" t="s">
         <v>314</v>
       </c>
@@ -6535,7 +6530,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" customHeight="1" spans="1:5">
       <c r="A80" s="1" t="s">
         <v>318</v>
       </c>
@@ -6552,7 +6547,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" customHeight="1" spans="1:5">
       <c r="A81" s="1" t="s">
         <v>323</v>
       </c>
@@ -6569,7 +6564,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" customHeight="1" spans="1:5">
       <c r="A82" s="1" t="s">
         <v>327</v>
       </c>
@@ -6586,7 +6581,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" customHeight="1" spans="1:5">
       <c r="A83" s="1" t="s">
         <v>331</v>
       </c>
@@ -6603,7 +6598,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" customHeight="1" spans="1:5">
       <c r="A84" s="1" t="s">
         <v>335</v>
       </c>
@@ -6620,7 +6615,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" customHeight="1" spans="1:5">
       <c r="A85" s="1" t="s">
         <v>339</v>
       </c>
@@ -6637,7 +6632,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" customHeight="1" spans="1:5">
       <c r="A86" s="1" t="s">
         <v>343</v>
       </c>
@@ -6654,7 +6649,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" customHeight="1" spans="1:5">
       <c r="A87" s="1" t="s">
         <v>347</v>
       </c>
@@ -6671,7 +6666,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" customHeight="1" spans="1:5">
       <c r="A88" s="1" t="s">
         <v>351</v>
       </c>
@@ -6688,7 +6683,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" customHeight="1" spans="1:5">
       <c r="A89" s="1" t="s">
         <v>355</v>
       </c>
@@ -6705,7 +6700,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" customHeight="1" spans="1:5">
       <c r="A90" s="1" t="s">
         <v>359</v>
       </c>
@@ -6722,8 +6717,8 @@
         <v>362</v>
       </c>
     </row>
-    <row r="91" ht="13.5" spans="1:5">
-      <c r="A91" s="1" t="s">
+    <row r="91" customHeight="1" spans="1:5">
+      <c r="A91" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B91" t="s">
@@ -6739,7 +6734,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" customHeight="1" spans="1:5">
       <c r="A92" s="1" t="s">
         <v>366</v>
       </c>
@@ -6756,7 +6751,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" customHeight="1" spans="1:5">
       <c r="A93" s="1" t="s">
         <v>370</v>
       </c>
@@ -6773,7 +6768,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" customHeight="1" spans="1:5">
       <c r="A94" s="1" t="s">
         <v>374</v>
       </c>
@@ -6790,7 +6785,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" customHeight="1" spans="1:5">
       <c r="A95" s="1" t="s">
         <v>378</v>
       </c>
@@ -6807,7 +6802,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" customHeight="1" spans="1:5">
       <c r="A96" s="1" t="s">
         <v>382</v>
       </c>
@@ -6824,7 +6819,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" customHeight="1" spans="1:5">
       <c r="A97" s="1" t="s">
         <v>386</v>
       </c>
@@ -6841,7 +6836,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" customHeight="1" spans="1:5">
       <c r="A98" s="1" t="s">
         <v>390</v>
       </c>
@@ -6858,7 +6853,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" customHeight="1" spans="1:5">
       <c r="A99" s="1" t="s">
         <v>394</v>
       </c>
@@ -6875,7 +6870,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" customHeight="1" spans="1:5">
       <c r="A100" s="1" t="s">
         <v>398</v>
       </c>
@@ -6892,7 +6887,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" customHeight="1" spans="1:5">
       <c r="A101" s="1" t="s">
         <v>402</v>
       </c>
@@ -6909,7 +6904,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" customHeight="1" spans="1:5">
       <c r="A102" s="1" t="s">
         <v>406</v>
       </c>
@@ -6926,7 +6921,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" customHeight="1" spans="1:5">
       <c r="A103" s="1" t="s">
         <v>410</v>
       </c>
@@ -6943,7 +6938,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" customHeight="1" spans="1:5">
       <c r="A104" s="1" t="s">
         <v>414</v>
       </c>
@@ -6960,7 +6955,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" customHeight="1" spans="1:5">
       <c r="A105" s="1" t="s">
         <v>418</v>
       </c>
@@ -6977,7 +6972,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" customHeight="1" spans="1:5">
       <c r="A106" s="1" t="s">
         <v>422</v>
       </c>
@@ -6994,7 +6989,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" customHeight="1" spans="1:5">
       <c r="A107" s="1" t="s">
         <v>426</v>
       </c>
@@ -7011,7 +7006,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" customHeight="1" spans="1:5">
       <c r="A108" s="1" t="s">
         <v>430</v>
       </c>
@@ -7028,7 +7023,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" customHeight="1" spans="1:5">
       <c r="A109" s="1" t="s">
         <v>434</v>
       </c>
@@ -7045,7 +7040,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" customHeight="1" spans="1:5">
       <c r="A110" s="1" t="s">
         <v>438</v>
       </c>
@@ -7062,7 +7057,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" customHeight="1" spans="1:5">
       <c r="A111" s="1" t="s">
         <v>442</v>
       </c>
@@ -7079,7 +7074,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" customHeight="1" spans="1:5">
       <c r="A112" s="1" t="s">
         <v>446</v>
       </c>
@@ -7096,7 +7091,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" customHeight="1" spans="1:5">
       <c r="A113" s="1" t="s">
         <v>450</v>
       </c>
@@ -7113,7 +7108,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" customHeight="1" spans="1:5">
       <c r="A114" s="1" t="s">
         <v>454</v>
       </c>
@@ -7130,7 +7125,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" customHeight="1" spans="1:5">
       <c r="A115" s="1" t="s">
         <v>458</v>
       </c>
@@ -7147,7 +7142,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" customHeight="1" spans="1:5">
       <c r="A116" s="1" t="s">
         <v>463</v>
       </c>
@@ -7164,7 +7159,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" customHeight="1" spans="1:5">
       <c r="A117" s="1" t="s">
         <v>467</v>
       </c>
@@ -7181,7 +7176,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" customHeight="1" spans="1:5">
       <c r="A118" s="1" t="s">
         <v>471</v>
       </c>
@@ -7198,7 +7193,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" customHeight="1" spans="1:5">
       <c r="A119" s="1" t="s">
         <v>475</v>
       </c>
@@ -7215,7 +7210,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" customHeight="1" spans="1:5">
       <c r="A120" s="1" t="s">
         <v>479</v>
       </c>
@@ -7232,7 +7227,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" customHeight="1" spans="1:5">
       <c r="A121" s="1" t="s">
         <v>484</v>
       </c>
@@ -7249,7 +7244,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" customHeight="1" spans="1:5">
       <c r="A122" s="1" t="s">
         <v>488</v>
       </c>
@@ -7266,7 +7261,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" customHeight="1" spans="1:5">
       <c r="A123" s="1" t="s">
         <v>492</v>
       </c>
@@ -7283,7 +7278,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" customHeight="1" spans="1:5">
       <c r="A124" s="1" t="s">
         <v>497</v>
       </c>
@@ -7300,7 +7295,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" customHeight="1" spans="1:5">
       <c r="A125" s="1" t="s">
         <v>501</v>
       </c>
@@ -7317,7 +7312,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="126" spans="1:5">
+    <row r="126" customHeight="1" spans="1:5">
       <c r="A126" s="1" t="s">
         <v>505</v>
       </c>
@@ -7334,7 +7329,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" customHeight="1" spans="1:5">
       <c r="A127" s="1" t="s">
         <v>509</v>
       </c>
@@ -7351,7 +7346,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" customHeight="1" spans="1:5">
       <c r="A128" s="1" t="s">
         <v>513</v>
       </c>
@@ -7368,7 +7363,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" customHeight="1" spans="1:5">
       <c r="A129" s="1" t="s">
         <v>517</v>
       </c>
@@ -7385,7 +7380,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" customHeight="1" spans="1:5">
       <c r="A130" s="1" t="s">
         <v>521</v>
       </c>
@@ -7402,7 +7397,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" customHeight="1" spans="1:5">
       <c r="A131" s="1" t="s">
         <v>525</v>
       </c>
@@ -7419,7 +7414,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" customHeight="1" spans="1:5">
       <c r="A132" s="1" t="s">
         <v>529</v>
       </c>
@@ -7436,7 +7431,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" customHeight="1" spans="1:5">
       <c r="A133" s="1" t="s">
         <v>533</v>
       </c>
@@ -7453,7 +7448,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" customHeight="1" spans="1:5">
       <c r="A134" s="1" t="s">
         <v>537</v>
       </c>
@@ -7470,7 +7465,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" customHeight="1" spans="1:5">
       <c r="A135" s="1" t="s">
         <v>541</v>
       </c>
@@ -7487,7 +7482,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" customHeight="1" spans="1:5">
       <c r="A136" s="1" t="s">
         <v>545</v>
       </c>
@@ -7504,7 +7499,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" customHeight="1" spans="1:5">
       <c r="A137" s="1" t="s">
         <v>549</v>
       </c>
@@ -7521,7 +7516,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" customHeight="1" spans="1:5">
       <c r="A138" s="1" t="s">
         <v>553</v>
       </c>
@@ -7538,7 +7533,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" customHeight="1" spans="1:5">
       <c r="A139" s="1" t="s">
         <v>557</v>
       </c>
@@ -7555,7 +7550,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" customHeight="1" spans="1:5">
       <c r="A140" s="1" t="s">
         <v>561</v>
       </c>
@@ -7572,7 +7567,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" customHeight="1" spans="1:5">
       <c r="A141" s="1" t="s">
         <v>565</v>
       </c>
@@ -7589,7 +7584,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" customHeight="1" spans="1:5">
       <c r="A142" s="1" t="s">
         <v>569</v>
       </c>
@@ -7606,7 +7601,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" customHeight="1" spans="1:5">
       <c r="A143" s="1" t="s">
         <v>573</v>
       </c>
@@ -7623,7 +7618,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" customHeight="1" spans="1:5">
       <c r="A144" s="1" t="s">
         <v>577</v>
       </c>
@@ -7640,7 +7635,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" customHeight="1" spans="1:5">
       <c r="A145" s="1" t="s">
         <v>581</v>
       </c>
@@ -7657,7 +7652,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" customHeight="1" spans="1:5">
       <c r="A146" s="1" t="s">
         <v>585</v>
       </c>
@@ -7674,7 +7669,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" customHeight="1" spans="1:5">
       <c r="A147" s="1" t="s">
         <v>589</v>
       </c>
@@ -7691,7 +7686,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" customHeight="1" spans="1:5">
       <c r="A148" s="1" t="s">
         <v>593</v>
       </c>
@@ -7708,7 +7703,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" customHeight="1" spans="1:5">
       <c r="A149" s="1" t="s">
         <v>597</v>
       </c>
@@ -7725,7 +7720,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" customHeight="1" spans="1:5">
       <c r="A150" s="1" t="s">
         <v>601</v>
       </c>
@@ -7742,7 +7737,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" customHeight="1" spans="1:5">
       <c r="A151" s="1" t="s">
         <v>605</v>
       </c>
@@ -7759,7 +7754,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" customHeight="1" spans="1:5">
       <c r="A152" s="1" t="s">
         <v>609</v>
       </c>
@@ -7776,7 +7771,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" customHeight="1" spans="1:5">
       <c r="A153" s="1" t="s">
         <v>613</v>
       </c>
@@ -7793,7 +7788,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" customHeight="1" spans="1:5">
       <c r="A154" s="1" t="s">
         <v>617</v>
       </c>
@@ -7810,7 +7805,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" customHeight="1" spans="1:5">
       <c r="A155" s="1" t="s">
         <v>621</v>
       </c>
@@ -7827,7 +7822,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" customHeight="1" spans="1:5">
       <c r="A156" s="1" t="s">
         <v>625</v>
       </c>
@@ -7844,7 +7839,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" customHeight="1" spans="1:5">
       <c r="A157" s="1" t="s">
         <v>629</v>
       </c>
@@ -7861,7 +7856,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" customHeight="1" spans="1:5">
       <c r="A158" s="1" t="s">
         <v>633</v>
       </c>
@@ -7878,7 +7873,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" customHeight="1" spans="1:5">
       <c r="A159" s="1" t="s">
         <v>637</v>
       </c>
@@ -7895,7 +7890,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" customHeight="1" spans="1:5">
       <c r="A160" s="1" t="s">
         <v>641</v>
       </c>
@@ -7912,7 +7907,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" customHeight="1" spans="1:5">
       <c r="A161" s="1" t="s">
         <v>645</v>
       </c>
@@ -7929,7 +7924,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" customHeight="1" spans="1:5">
       <c r="A162" s="1" t="s">
         <v>649</v>
       </c>
@@ -7946,7 +7941,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" customHeight="1" spans="1:5">
       <c r="A163" s="1" t="s">
         <v>653</v>
       </c>
@@ -7963,7 +7958,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" customHeight="1" spans="1:5">
       <c r="A164" s="1" t="s">
         <v>657</v>
       </c>
@@ -7980,7 +7975,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" customHeight="1" spans="1:5">
       <c r="A165" s="1" t="s">
         <v>661</v>
       </c>
@@ -7997,7 +7992,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" customHeight="1" spans="1:5">
       <c r="A166" s="1" t="s">
         <v>665</v>
       </c>
@@ -8014,7 +8009,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" customHeight="1" spans="1:5">
       <c r="A167" s="1" t="s">
         <v>669</v>
       </c>
@@ -8031,7 +8026,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" customHeight="1" spans="1:5">
       <c r="A168" s="1" t="s">
         <v>673</v>
       </c>
@@ -8048,7 +8043,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" customHeight="1" spans="1:5">
       <c r="A169" s="1" t="s">
         <v>677</v>
       </c>
@@ -8065,7 +8060,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" customHeight="1" spans="1:5">
       <c r="A170" s="1" t="s">
         <v>681</v>
       </c>
@@ -8082,7 +8077,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="171" spans="1:5">
+    <row r="171" customHeight="1" spans="1:5">
       <c r="A171" s="1" t="s">
         <v>685</v>
       </c>
@@ -8099,7 +8094,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" customHeight="1" spans="1:5">
       <c r="A172" s="1" t="s">
         <v>689</v>
       </c>
@@ -8116,7 +8111,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" customHeight="1" spans="1:5">
       <c r="A173" s="1" t="s">
         <v>693</v>
       </c>
@@ -8133,7 +8128,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" customHeight="1" spans="1:5">
       <c r="A174" s="1" t="s">
         <v>697</v>
       </c>
@@ -8150,7 +8145,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="175" spans="1:5">
+    <row r="175" customHeight="1" spans="1:5">
       <c r="A175" s="1" t="s">
         <v>701</v>
       </c>
@@ -8167,7 +8162,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="176" spans="1:5">
+    <row r="176" customHeight="1" spans="1:5">
       <c r="A176" s="1" t="s">
         <v>705</v>
       </c>
@@ -8184,7 +8179,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="177" spans="1:5">
+    <row r="177" customHeight="1" spans="1:5">
       <c r="A177" s="1" t="s">
         <v>709</v>
       </c>
@@ -8201,7 +8196,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="178" spans="1:5">
+    <row r="178" customHeight="1" spans="1:5">
       <c r="A178" s="1" t="s">
         <v>713</v>
       </c>
@@ -8218,7 +8213,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="179" spans="1:5">
+    <row r="179" customHeight="1" spans="1:5">
       <c r="A179" s="1" t="s">
         <v>717</v>
       </c>
@@ -8235,7 +8230,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="180" spans="1:5">
+    <row r="180" customHeight="1" spans="1:5">
       <c r="A180" s="1" t="s">
         <v>721</v>
       </c>
@@ -8252,7 +8247,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="181" spans="1:5">
+    <row r="181" customHeight="1" spans="1:5">
       <c r="A181" s="1" t="s">
         <v>725</v>
       </c>
@@ -8269,7 +8264,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="182" spans="1:5">
+    <row r="182" customHeight="1" spans="1:5">
       <c r="A182" s="1" t="s">
         <v>729</v>
       </c>
@@ -8286,7 +8281,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="183" spans="1:5">
+    <row r="183" customHeight="1" spans="1:5">
       <c r="A183" s="1" t="s">
         <v>733</v>
       </c>
@@ -8303,7 +8298,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="184" spans="1:5">
+    <row r="184" customHeight="1" spans="1:5">
       <c r="A184" s="1" t="s">
         <v>737</v>
       </c>
@@ -8320,7 +8315,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="185" spans="1:5">
+    <row r="185" customHeight="1" spans="1:5">
       <c r="A185" s="1" t="s">
         <v>741</v>
       </c>
@@ -8337,7 +8332,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="186" spans="1:5">
+    <row r="186" customHeight="1" spans="1:5">
       <c r="A186" s="1" t="s">
         <v>745</v>
       </c>
@@ -8354,7 +8349,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="187" spans="1:5">
+    <row r="187" customHeight="1" spans="1:5">
       <c r="A187" s="1" t="s">
         <v>750</v>
       </c>
@@ -8371,7 +8366,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="188" spans="1:5">
+    <row r="188" customHeight="1" spans="1:5">
       <c r="A188" s="1" t="s">
         <v>754</v>
       </c>
@@ -8388,7 +8383,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="189" spans="1:5">
+    <row r="189" customHeight="1" spans="1:5">
       <c r="A189" s="1" t="s">
         <v>758</v>
       </c>
@@ -8405,7 +8400,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="190" spans="1:5">
+    <row r="190" customHeight="1" spans="1:5">
       <c r="A190" s="1" t="s">
         <v>762</v>
       </c>
@@ -8422,7 +8417,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="191" spans="1:5">
+    <row r="191" customHeight="1" spans="1:5">
       <c r="A191" s="1" t="s">
         <v>766</v>
       </c>
@@ -8439,7 +8434,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="192" spans="1:5">
+    <row r="192" customHeight="1" spans="1:5">
       <c r="A192" s="1" t="s">
         <v>770</v>
       </c>
@@ -8456,7 +8451,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="193" spans="1:5">
+    <row r="193" customHeight="1" spans="1:5">
       <c r="A193" s="1" t="s">
         <v>774</v>
       </c>
@@ -8473,7 +8468,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="194" spans="1:5">
+    <row r="194" customHeight="1" spans="1:5">
       <c r="A194" s="1" t="s">
         <v>778</v>
       </c>
@@ -8490,7 +8485,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="195" spans="1:5">
+    <row r="195" customHeight="1" spans="1:5">
       <c r="A195" s="1" t="s">
         <v>782</v>
       </c>
@@ -8507,7 +8502,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="196" spans="1:5">
+    <row r="196" customHeight="1" spans="1:5">
       <c r="A196" s="1" t="s">
         <v>786</v>
       </c>
@@ -8524,7 +8519,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="197" spans="1:5">
+    <row r="197" customHeight="1" spans="1:5">
       <c r="A197" s="1" t="s">
         <v>790</v>
       </c>
@@ -8541,7 +8536,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="198" spans="1:5">
+    <row r="198" customHeight="1" spans="1:5">
       <c r="A198" s="1" t="s">
         <v>794</v>
       </c>
@@ -8558,7 +8553,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="199" spans="1:5">
+    <row r="199" customHeight="1" spans="1:5">
       <c r="A199" s="1" t="s">
         <v>799</v>
       </c>
@@ -8575,7 +8570,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="200" spans="1:5">
+    <row r="200" customHeight="1" spans="1:5">
       <c r="A200" s="1" t="s">
         <v>803</v>
       </c>
@@ -8592,7 +8587,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="201" spans="1:5">
+    <row r="201" customHeight="1" spans="1:5">
       <c r="A201" s="1" t="s">
         <v>807</v>
       </c>
@@ -8609,7 +8604,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="202" spans="1:5">
+    <row r="202" customHeight="1" spans="1:5">
       <c r="A202" s="1" t="s">
         <v>811</v>
       </c>
@@ -8626,7 +8621,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="203" spans="1:5">
+    <row r="203" customHeight="1" spans="1:5">
       <c r="A203" s="1" t="s">
         <v>815</v>
       </c>
@@ -8643,7 +8638,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="204" spans="1:5">
+    <row r="204" customHeight="1" spans="1:5">
       <c r="A204" s="1" t="s">
         <v>819</v>
       </c>
@@ -8660,7 +8655,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="205" spans="1:5">
+    <row r="205" customHeight="1" spans="1:5">
       <c r="A205" s="1" t="s">
         <v>823</v>
       </c>
@@ -8677,7 +8672,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="206" spans="1:5">
+    <row r="206" customHeight="1" spans="1:5">
       <c r="A206" s="1" t="s">
         <v>827</v>
       </c>
@@ -8694,7 +8689,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="207" spans="1:5">
+    <row r="207" customHeight="1" spans="1:5">
       <c r="A207" s="1" t="s">
         <v>831</v>
       </c>
@@ -8711,7 +8706,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="208" spans="1:5">
+    <row r="208" customHeight="1" spans="1:5">
       <c r="A208" s="1" t="s">
         <v>835</v>
       </c>
@@ -8728,7 +8723,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="209" spans="1:5">
+    <row r="209" customHeight="1" spans="1:5">
       <c r="A209" s="1" t="s">
         <v>839</v>
       </c>
@@ -8745,7 +8740,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="210" spans="1:5">
+    <row r="210" customHeight="1" spans="1:5">
       <c r="A210" s="1" t="s">
         <v>843</v>
       </c>
@@ -8762,7 +8757,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="211" spans="1:5">
+    <row r="211" customHeight="1" spans="1:5">
       <c r="A211" s="1" t="s">
         <v>847</v>
       </c>
@@ -8779,7 +8774,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="212" spans="1:5">
+    <row r="212" customHeight="1" spans="1:5">
       <c r="A212" s="1" t="s">
         <v>851</v>
       </c>
@@ -8796,7 +8791,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="213" spans="1:5">
+    <row r="213" customHeight="1" spans="1:5">
       <c r="A213" s="1" t="s">
         <v>855</v>
       </c>
@@ -8813,7 +8808,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="214" spans="1:5">
+    <row r="214" customHeight="1" spans="1:5">
       <c r="A214" s="1" t="s">
         <v>859</v>
       </c>
@@ -8830,7 +8825,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="215" spans="1:5">
+    <row r="215" customHeight="1" spans="1:5">
       <c r="A215" s="1" t="s">
         <v>863</v>
       </c>
@@ -8847,7 +8842,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="216" spans="1:5">
+    <row r="216" customHeight="1" spans="1:5">
       <c r="A216" s="1" t="s">
         <v>867</v>
       </c>
@@ -8864,7 +8859,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="217" spans="1:5">
+    <row r="217" customHeight="1" spans="1:5">
       <c r="A217" s="1" t="s">
         <v>871</v>
       </c>
@@ -8881,7 +8876,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="218" spans="1:5">
+    <row r="218" customHeight="1" spans="1:5">
       <c r="A218" s="1" t="s">
         <v>875</v>
       </c>
@@ -8898,7 +8893,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="219" spans="1:5">
+    <row r="219" customHeight="1" spans="1:5">
       <c r="A219" s="1" t="s">
         <v>880</v>
       </c>
@@ -8915,7 +8910,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="220" spans="1:5">
+    <row r="220" customHeight="1" spans="1:5">
       <c r="A220" s="1" t="s">
         <v>884</v>
       </c>
@@ -8932,7 +8927,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="221" spans="1:5">
+    <row r="221" customHeight="1" spans="1:5">
       <c r="A221" s="1" t="s">
         <v>888</v>
       </c>
@@ -8949,7 +8944,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="222" spans="1:5">
+    <row r="222" customHeight="1" spans="1:5">
       <c r="A222" s="1" t="s">
         <v>892</v>
       </c>
@@ -8966,7 +8961,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="223" spans="1:5">
+    <row r="223" customHeight="1" spans="1:5">
       <c r="A223" s="1" t="s">
         <v>896</v>
       </c>
@@ -8983,7 +8978,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="224" spans="1:5">
+    <row r="224" customHeight="1" spans="1:5">
       <c r="A224" s="1" t="s">
         <v>900</v>
       </c>
@@ -9000,7 +8995,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="225" spans="1:5">
+    <row r="225" customHeight="1" spans="1:5">
       <c r="A225" s="1" t="s">
         <v>904</v>
       </c>
@@ -9017,7 +9012,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="226" spans="1:5">
+    <row r="226" customHeight="1" spans="1:5">
       <c r="A226" s="1" t="s">
         <v>909</v>
       </c>
@@ -9034,7 +9029,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="227" spans="1:5">
+    <row r="227" customHeight="1" spans="1:5">
       <c r="A227" s="1" t="s">
         <v>913</v>
       </c>
@@ -9051,7 +9046,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="228" spans="1:5">
+    <row r="228" customHeight="1" spans="1:5">
       <c r="A228" s="1" t="s">
         <v>918</v>
       </c>
@@ -9068,7 +9063,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="229" spans="1:5">
+    <row r="229" customHeight="1" spans="1:5">
       <c r="A229" s="1" t="s">
         <v>923</v>
       </c>
@@ -9085,7 +9080,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="230" spans="1:5">
+    <row r="230" customHeight="1" spans="1:5">
       <c r="A230" s="1" t="s">
         <v>927</v>
       </c>
@@ -9102,7 +9097,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="231" spans="1:5">
+    <row r="231" customHeight="1" spans="1:5">
       <c r="A231" s="1" t="s">
         <v>931</v>
       </c>
@@ -9119,7 +9114,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="232" spans="1:5">
+    <row r="232" customHeight="1" spans="1:5">
       <c r="A232" s="1" t="s">
         <v>935</v>
       </c>
@@ -9136,7 +9131,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="233" spans="1:5">
+    <row r="233" customHeight="1" spans="1:5">
       <c r="A233" s="1" t="s">
         <v>939</v>
       </c>
@@ -9153,7 +9148,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="234" spans="1:5">
+    <row r="234" customHeight="1" spans="1:5">
       <c r="A234" s="1" t="s">
         <v>943</v>
       </c>
@@ -9170,7 +9165,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="235" spans="1:5">
+    <row r="235" customHeight="1" spans="1:5">
       <c r="A235" s="1" t="s">
         <v>947</v>
       </c>
@@ -9187,7 +9182,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="236" spans="1:5">
+    <row r="236" customHeight="1" spans="1:5">
       <c r="A236" s="1" t="s">
         <v>951</v>
       </c>
@@ -9204,7 +9199,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="237" spans="1:5">
+    <row r="237" customHeight="1" spans="1:5">
       <c r="A237" s="1" t="s">
         <v>955</v>
       </c>
@@ -9221,7 +9216,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="238" spans="1:5">
+    <row r="238" customHeight="1" spans="1:5">
       <c r="A238" s="1" t="s">
         <v>959</v>
       </c>
@@ -9238,7 +9233,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="239" spans="1:5">
+    <row r="239" customHeight="1" spans="1:5">
       <c r="A239" s="1" t="s">
         <v>963</v>
       </c>
@@ -9255,7 +9250,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="240" spans="1:5">
+    <row r="240" customHeight="1" spans="1:5">
       <c r="A240" s="1" t="s">
         <v>967</v>
       </c>
@@ -9272,7 +9267,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="241" spans="1:5">
+    <row r="241" customHeight="1" spans="1:5">
       <c r="A241" s="1" t="s">
         <v>971</v>
       </c>
@@ -9289,7 +9284,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="242" spans="1:5">
+    <row r="242" customHeight="1" spans="1:5">
       <c r="A242" s="1" t="s">
         <v>975</v>
       </c>
@@ -9306,7 +9301,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="243" spans="1:5">
+    <row r="243" customHeight="1" spans="1:5">
       <c r="A243" s="1" t="s">
         <v>979</v>
       </c>
@@ -9323,7 +9318,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="244" spans="1:5">
+    <row r="244" customHeight="1" spans="1:5">
       <c r="A244" s="1" t="s">
         <v>983</v>
       </c>
@@ -9340,7 +9335,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="245" spans="1:5">
+    <row r="245" customHeight="1" spans="1:5">
       <c r="A245" s="1" t="s">
         <v>987</v>
       </c>
@@ -9357,7 +9352,7 @@
         <v>991</v>
       </c>
     </row>
-    <row r="246" spans="1:5">
+    <row r="246" customHeight="1" spans="1:5">
       <c r="A246" s="1" t="s">
         <v>992</v>
       </c>
@@ -9374,7 +9369,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="247" spans="1:5">
+    <row r="247" customHeight="1" spans="1:5">
       <c r="A247" s="1" t="s">
         <v>997</v>
       </c>
@@ -9391,7 +9386,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="248" spans="1:5">
+    <row r="248" customHeight="1" spans="1:5">
       <c r="A248" s="1" t="s">
         <v>1001</v>
       </c>
@@ -9408,7 +9403,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="249" spans="1:5">
+    <row r="249" customHeight="1" spans="1:5">
       <c r="A249" s="1" t="s">
         <v>1005</v>
       </c>
@@ -9425,7 +9420,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="250" spans="1:5">
+    <row r="250" customHeight="1" spans="1:5">
       <c r="A250" s="1" t="s">
         <v>1009</v>
       </c>
@@ -9442,7 +9437,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="251" spans="1:5">
+    <row r="251" customHeight="1" spans="1:5">
       <c r="A251" s="1" t="s">
         <v>1013</v>
       </c>
@@ -9459,7 +9454,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="252" spans="1:5">
+    <row r="252" customHeight="1" spans="1:5">
       <c r="A252" s="1" t="s">
         <v>1017</v>
       </c>
@@ -9476,7 +9471,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="253" spans="1:5">
+    <row r="253" customHeight="1" spans="1:5">
       <c r="A253" s="1" t="s">
         <v>1021</v>
       </c>
@@ -9493,7 +9488,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="254" spans="1:5">
+    <row r="254" customHeight="1" spans="1:5">
       <c r="A254" s="1" t="s">
         <v>1025</v>
       </c>
@@ -9510,7 +9505,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="255" spans="1:5">
+    <row r="255" customHeight="1" spans="1:5">
       <c r="A255" s="1" t="s">
         <v>1029</v>
       </c>
@@ -9527,7 +9522,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="256" spans="1:5">
+    <row r="256" customHeight="1" spans="1:5">
       <c r="A256" s="1" t="s">
         <v>1033</v>
       </c>
@@ -9544,7 +9539,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="257" spans="1:5">
+    <row r="257" customHeight="1" spans="1:5">
       <c r="A257" s="1" t="s">
         <v>1038</v>
       </c>
@@ -9561,7 +9556,7 @@
         <v>1041</v>
       </c>
     </row>
-    <row r="258" spans="1:5">
+    <row r="258" customHeight="1" spans="1:5">
       <c r="A258" s="1" t="s">
         <v>1042</v>
       </c>
@@ -9578,7 +9573,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="259" spans="1:5">
+    <row r="259" customHeight="1" spans="1:5">
       <c r="A259" s="1" t="s">
         <v>1046</v>
       </c>
@@ -9595,7 +9590,7 @@
         <v>1049</v>
       </c>
     </row>
-    <row r="260" spans="1:5">
+    <row r="260" customHeight="1" spans="1:5">
       <c r="A260" s="1" t="s">
         <v>1050</v>
       </c>
@@ -9612,7 +9607,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="261" spans="1:5">
+    <row r="261" customHeight="1" spans="1:5">
       <c r="A261" s="1" t="s">
         <v>1054</v>
       </c>
@@ -9629,7 +9624,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="262" spans="1:5">
+    <row r="262" customHeight="1" spans="1:5">
       <c r="A262" s="1" t="s">
         <v>1058</v>
       </c>
@@ -9646,7 +9641,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="263" spans="1:5">
+    <row r="263" customHeight="1" spans="1:5">
       <c r="A263" s="1" t="s">
         <v>1062</v>
       </c>
@@ -9663,7 +9658,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="264" spans="1:5">
+    <row r="264" customHeight="1" spans="1:5">
       <c r="A264" s="1" t="s">
         <v>1066</v>
       </c>
@@ -9680,7 +9675,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="265" spans="1:5">
+    <row r="265" customHeight="1" spans="1:5">
       <c r="A265" s="1" t="s">
         <v>1070</v>
       </c>
@@ -9697,7 +9692,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="266" spans="1:5">
+    <row r="266" customHeight="1" spans="1:5">
       <c r="A266" s="1" t="s">
         <v>1074</v>
       </c>
@@ -9714,7 +9709,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="267" spans="1:5">
+    <row r="267" customHeight="1" spans="1:5">
       <c r="A267" s="1" t="s">
         <v>1078</v>
       </c>
@@ -9731,7 +9726,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="268" spans="1:5">
+    <row r="268" customHeight="1" spans="1:5">
       <c r="A268" s="1" t="s">
         <v>1082</v>
       </c>
@@ -9748,7 +9743,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="269" spans="1:5">
+    <row r="269" customHeight="1" spans="1:5">
       <c r="A269" s="1" t="s">
         <v>1087</v>
       </c>
@@ -9765,7 +9760,7 @@
         <v>1091</v>
       </c>
     </row>
-    <row r="270" spans="1:5">
+    <row r="270" customHeight="1" spans="1:5">
       <c r="A270" s="1" t="s">
         <v>1092</v>
       </c>
@@ -9782,7 +9777,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="271" spans="1:5">
+    <row r="271" customHeight="1" spans="1:5">
       <c r="A271" s="1" t="s">
         <v>1097</v>
       </c>
@@ -9799,7 +9794,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="272" spans="1:5">
+    <row r="272" customHeight="1" spans="1:5">
       <c r="A272" s="1" t="s">
         <v>1101</v>
       </c>
@@ -9816,7 +9811,7 @@
         <v>1104</v>
       </c>
     </row>
-    <row r="273" spans="1:5">
+    <row r="273" customHeight="1" spans="1:5">
       <c r="A273" s="1" t="s">
         <v>1105</v>
       </c>
@@ -9833,7 +9828,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="274" spans="1:5">
+    <row r="274" customHeight="1" spans="1:5">
       <c r="A274" s="1" t="s">
         <v>1109</v>
       </c>
@@ -9850,7 +9845,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="275" spans="1:5">
+    <row r="275" customHeight="1" spans="1:5">
       <c r="A275" s="1" t="s">
         <v>1113</v>
       </c>
@@ -9867,7 +9862,7 @@
         <v>1116</v>
       </c>
     </row>
-    <row r="276" spans="1:5">
+    <row r="276" customHeight="1" spans="1:5">
       <c r="A276" s="1" t="s">
         <v>1117</v>
       </c>
@@ -9884,7 +9879,7 @@
         <v>1120</v>
       </c>
     </row>
-    <row r="277" spans="1:5">
+    <row r="277" customHeight="1" spans="1:5">
       <c r="A277" s="1" t="s">
         <v>1121</v>
       </c>
@@ -9901,7 +9896,7 @@
         <v>1124</v>
       </c>
     </row>
-    <row r="278" spans="1:5">
+    <row r="278" customHeight="1" spans="1:5">
       <c r="A278" s="1" t="s">
         <v>1125</v>
       </c>
@@ -9918,7 +9913,7 @@
         <v>1128</v>
       </c>
     </row>
-    <row r="279" spans="1:5">
+    <row r="279" customHeight="1" spans="1:5">
       <c r="A279" s="1" t="s">
         <v>1129</v>
       </c>
@@ -9935,7 +9930,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="280" spans="1:5">
+    <row r="280" customHeight="1" spans="1:5">
       <c r="A280" s="1" t="s">
         <v>1133</v>
       </c>
@@ -9952,7 +9947,7 @@
         <v>1136</v>
       </c>
     </row>
-    <row r="281" spans="1:5">
+    <row r="281" customHeight="1" spans="1:5">
       <c r="A281" s="1" t="s">
         <v>1137</v>
       </c>
@@ -9969,7 +9964,7 @@
         <v>1140</v>
       </c>
     </row>
-    <row r="282" spans="1:5">
+    <row r="282" customHeight="1" spans="1:5">
       <c r="A282" s="1" t="s">
         <v>1141</v>
       </c>
@@ -9986,7 +9981,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="283" spans="1:5">
+    <row r="283" customHeight="1" spans="1:5">
       <c r="A283" s="1" t="s">
         <v>1146</v>
       </c>
@@ -10003,7 +9998,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="284" spans="1:5">
+    <row r="284" customHeight="1" spans="1:5">
       <c r="A284" s="1" t="s">
         <v>1150</v>
       </c>
@@ -10020,7 +10015,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="285" spans="1:5">
+    <row r="285" customHeight="1" spans="1:5">
       <c r="A285" s="1" t="s">
         <v>1155</v>
       </c>
@@ -10037,7 +10032,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="286" spans="1:5">
+    <row r="286" customHeight="1" spans="1:5">
       <c r="A286" s="1" t="s">
         <v>1160</v>
       </c>
@@ -10054,7 +10049,7 @@
         <v>1163</v>
       </c>
     </row>
-    <row r="287" spans="1:5">
+    <row r="287" customHeight="1" spans="1:5">
       <c r="A287" s="1" t="s">
         <v>1164</v>
       </c>
@@ -10071,7 +10066,7 @@
         <v>1168</v>
       </c>
     </row>
-    <row r="288" spans="1:5">
+    <row r="288" customHeight="1" spans="1:5">
       <c r="A288" s="1" t="s">
         <v>1169</v>
       </c>
@@ -10088,7 +10083,7 @@
         <v>1172</v>
       </c>
     </row>
-    <row r="289" spans="1:5">
+    <row r="289" customHeight="1" spans="1:5">
       <c r="A289" s="1" t="s">
         <v>1173</v>
       </c>
@@ -10105,7 +10100,7 @@
         <v>1177</v>
       </c>
     </row>
-    <row r="290" spans="1:5">
+    <row r="290" customHeight="1" spans="1:5">
       <c r="A290" s="1" t="s">
         <v>1178</v>
       </c>
@@ -10122,7 +10117,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="291" spans="1:5">
+    <row r="291" customHeight="1" spans="1:5">
       <c r="A291" s="1" t="s">
         <v>1182</v>
       </c>
@@ -10139,7 +10134,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="292" spans="1:5">
+    <row r="292" customHeight="1" spans="1:5">
       <c r="A292" s="1" t="s">
         <v>1186</v>
       </c>
@@ -10156,7 +10151,7 @@
         <v>1189</v>
       </c>
     </row>
-    <row r="293" spans="1:5">
+    <row r="293" customHeight="1" spans="1:5">
       <c r="A293" s="1" t="s">
         <v>1190</v>
       </c>
@@ -10173,7 +10168,7 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="294" spans="1:5">
+    <row r="294" customHeight="1" spans="1:5">
       <c r="A294" s="1" t="s">
         <v>1195</v>
       </c>
@@ -10190,7 +10185,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="295" spans="1:5">
+    <row r="295" customHeight="1" spans="1:5">
       <c r="A295" s="1" t="s">
         <v>1199</v>
       </c>
@@ -10207,7 +10202,7 @@
         <v>1202</v>
       </c>
     </row>
-    <row r="296" spans="1:5">
+    <row r="296" customHeight="1" spans="1:5">
       <c r="A296" s="1" t="s">
         <v>1203</v>
       </c>
@@ -10224,7 +10219,7 @@
         <v>1206</v>
       </c>
     </row>
-    <row r="297" spans="1:5">
+    <row r="297" customHeight="1" spans="1:5">
       <c r="A297" s="1" t="s">
         <v>1207</v>
       </c>
@@ -10241,7 +10236,7 @@
         <v>1210</v>
       </c>
     </row>
-    <row r="298" spans="1:5">
+    <row r="298" customHeight="1" spans="1:5">
       <c r="A298" s="1" t="s">
         <v>1211</v>
       </c>
@@ -10258,7 +10253,7 @@
         <v>1214</v>
       </c>
     </row>
-    <row r="299" spans="1:5">
+    <row r="299" customHeight="1" spans="1:5">
       <c r="A299" s="1" t="s">
         <v>1215</v>
       </c>
@@ -10275,7 +10270,7 @@
         <v>1218</v>
       </c>
     </row>
-    <row r="300" spans="1:5">
+    <row r="300" customHeight="1" spans="1:5">
       <c r="A300" s="1" t="s">
         <v>1219</v>
       </c>
@@ -10292,7 +10287,7 @@
         <v>1221</v>
       </c>
     </row>
-    <row r="301" spans="1:5">
+    <row r="301" customHeight="1" spans="1:5">
       <c r="A301" s="1" t="s">
         <v>1222</v>
       </c>
@@ -10309,7 +10304,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="302" spans="1:5">
+    <row r="302" customHeight="1" spans="1:5">
       <c r="A302" s="1" t="s">
         <v>1225</v>
       </c>
@@ -10326,7 +10321,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="303" spans="1:5">
+    <row r="303" customHeight="1" spans="1:5">
       <c r="A303" s="1" t="s">
         <v>1228</v>
       </c>
@@ -10343,7 +10338,7 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="304" spans="1:5">
+    <row r="304" customHeight="1" spans="1:5">
       <c r="A304" s="1" t="s">
         <v>1231</v>
       </c>
@@ -10360,7 +10355,7 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="305" spans="1:5">
+    <row r="305" customHeight="1" spans="1:5">
       <c r="A305" s="1" t="s">
         <v>1234</v>
       </c>
@@ -10377,7 +10372,7 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="306" spans="1:5">
+    <row r="306" customHeight="1" spans="1:5">
       <c r="A306" s="1" t="s">
         <v>1237</v>
       </c>
@@ -10394,7 +10389,7 @@
         <v>1239</v>
       </c>
     </row>
-    <row r="307" spans="1:5">
+    <row r="307" customHeight="1" spans="1:5">
       <c r="A307" s="1" t="s">
         <v>1240</v>
       </c>
@@ -10411,7 +10406,7 @@
         <v>1242</v>
       </c>
     </row>
-    <row r="308" spans="1:5">
+    <row r="308" customHeight="1" spans="1:5">
       <c r="A308" s="1" t="s">
         <v>1243</v>
       </c>
@@ -10428,7 +10423,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="309" spans="1:5">
+    <row r="309" customHeight="1" spans="1:5">
       <c r="A309" s="1" t="s">
         <v>1246</v>
       </c>
@@ -10445,7 +10440,7 @@
         <v>1248</v>
       </c>
     </row>
-    <row r="310" spans="1:5">
+    <row r="310" customHeight="1" spans="1:5">
       <c r="A310" s="1" t="s">
         <v>1249</v>
       </c>
@@ -10462,7 +10457,7 @@
         <v>1251</v>
       </c>
     </row>
-    <row r="311" spans="1:5">
+    <row r="311" customHeight="1" spans="1:5">
       <c r="A311" s="1" t="s">
         <v>1252</v>
       </c>
@@ -10479,7 +10474,7 @@
         <v>1254</v>
       </c>
     </row>
-    <row r="312" spans="1:5">
+    <row r="312" customHeight="1" spans="1:5">
       <c r="A312" s="1" t="s">
         <v>1255</v>
       </c>
@@ -10496,7 +10491,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="313" spans="1:5">
+    <row r="313" customHeight="1" spans="1:5">
       <c r="A313" s="1" t="s">
         <v>1258</v>
       </c>
@@ -10513,7 +10508,7 @@
         <v>1260</v>
       </c>
     </row>
-    <row r="314" spans="1:5">
+    <row r="314" customHeight="1" spans="1:5">
       <c r="A314" s="1" t="s">
         <v>1261</v>
       </c>
@@ -10530,7 +10525,7 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="315" spans="1:5">
+    <row r="315" customHeight="1" spans="1:5">
       <c r="A315" s="1" t="s">
         <v>1264</v>
       </c>
@@ -10547,7 +10542,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="316" spans="1:5">
+    <row r="316" customHeight="1" spans="1:5">
       <c r="A316" s="1" t="s">
         <v>1267</v>
       </c>
@@ -10564,7 +10559,7 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="317" spans="1:5">
+    <row r="317" customHeight="1" spans="1:5">
       <c r="A317" s="1" t="s">
         <v>1270</v>
       </c>
@@ -10581,7 +10576,7 @@
         <v>1272</v>
       </c>
     </row>
-    <row r="318" spans="1:5">
+    <row r="318" customHeight="1" spans="1:5">
       <c r="A318" s="1" t="s">
         <v>1273</v>
       </c>
@@ -10598,7 +10593,7 @@
         <v>1275</v>
       </c>
     </row>
-    <row r="319" spans="1:5">
+    <row r="319" customHeight="1" spans="1:5">
       <c r="A319" s="1" t="s">
         <v>1276</v>
       </c>
@@ -10615,7 +10610,7 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="320" spans="1:5">
+    <row r="320" customHeight="1" spans="1:5">
       <c r="A320" s="1" t="s">
         <v>1279</v>
       </c>
@@ -10632,7 +10627,7 @@
         <v>1281</v>
       </c>
     </row>
-    <row r="321" spans="1:5">
+    <row r="321" customHeight="1" spans="1:5">
       <c r="A321" s="1" t="s">
         <v>1282</v>
       </c>
@@ -10649,7 +10644,7 @@
         <v>1284</v>
       </c>
     </row>
-    <row r="322" spans="1:5">
+    <row r="322" customHeight="1" spans="1:5">
       <c r="A322" s="1" t="s">
         <v>1285</v>
       </c>
@@ -10666,7 +10661,7 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="323" spans="1:5">
+    <row r="323" customHeight="1" spans="1:5">
       <c r="A323" s="1" t="s">
         <v>1288</v>
       </c>
@@ -10683,7 +10678,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="324" spans="1:5">
+    <row r="324" customHeight="1" spans="1:5">
       <c r="A324" s="1" t="s">
         <v>1291</v>
       </c>
@@ -10700,7 +10695,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="325" spans="1:5">
+    <row r="325" customHeight="1" spans="1:5">
       <c r="A325" s="1" t="s">
         <v>1294</v>
       </c>
@@ -10717,7 +10712,7 @@
         <v>1296</v>
       </c>
     </row>
-    <row r="326" spans="1:5">
+    <row r="326" customHeight="1" spans="1:5">
       <c r="A326" s="1" t="s">
         <v>1297</v>
       </c>
@@ -10734,7 +10729,7 @@
         <v>1299</v>
       </c>
     </row>
-    <row r="327" spans="1:5">
+    <row r="327" customHeight="1" spans="1:5">
       <c r="A327" s="1" t="s">
         <v>1300</v>
       </c>
@@ -10751,7 +10746,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="328" spans="1:5">
+    <row r="328" customHeight="1" spans="1:5">
       <c r="A328" s="1" t="s">
         <v>1303</v>
       </c>
@@ -10768,7 +10763,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="329" spans="1:5">
+    <row r="329" customHeight="1" spans="1:5">
       <c r="A329" s="1" t="s">
         <v>1306</v>
       </c>
@@ -10785,7 +10780,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="330" spans="1:5">
+    <row r="330" customHeight="1" spans="1:5">
       <c r="A330" s="1" t="s">
         <v>1309</v>
       </c>
@@ -10802,7 +10797,7 @@
         <v>1311</v>
       </c>
     </row>
-    <row r="331" spans="1:5">
+    <row r="331" customHeight="1" spans="1:5">
       <c r="A331" s="1" t="s">
         <v>1312</v>
       </c>
@@ -10819,7 +10814,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="332" spans="1:5">
+    <row r="332" customHeight="1" spans="1:5">
       <c r="A332" s="1" t="s">
         <v>1315</v>
       </c>
@@ -10836,7 +10831,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="333" spans="1:5">
+    <row r="333" customHeight="1" spans="1:5">
       <c r="A333" s="1" t="s">
         <v>1318</v>
       </c>
@@ -10853,7 +10848,7 @@
         <v>1320</v>
       </c>
     </row>
-    <row r="334" spans="1:5">
+    <row r="334" customHeight="1" spans="1:5">
       <c r="A334" s="1" t="s">
         <v>1321</v>
       </c>
@@ -10870,7 +10865,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="335" spans="1:5">
+    <row r="335" customHeight="1" spans="1:5">
       <c r="A335" s="1" t="s">
         <v>1324</v>
       </c>
@@ -10887,7 +10882,7 @@
         <v>1326</v>
       </c>
     </row>
-    <row r="336" spans="1:5">
+    <row r="336" customHeight="1" spans="1:5">
       <c r="A336" s="1" t="s">
         <v>1327</v>
       </c>
@@ -10904,7 +10899,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="337" spans="1:5">
+    <row r="337" customHeight="1" spans="1:5">
       <c r="A337" s="1" t="s">
         <v>1330</v>
       </c>
@@ -10921,7 +10916,7 @@
         <v>1332</v>
       </c>
     </row>
-    <row r="338" spans="1:5">
+    <row r="338" customHeight="1" spans="1:5">
       <c r="A338" s="1" t="s">
         <v>1333</v>
       </c>
@@ -10938,7 +10933,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="339" spans="1:5">
+    <row r="339" customHeight="1" spans="1:5">
       <c r="A339" s="1" t="s">
         <v>1336</v>
       </c>
@@ -10955,7 +10950,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="340" spans="1:5">
+    <row r="340" customHeight="1" spans="1:5">
       <c r="A340" s="1" t="s">
         <v>1339</v>
       </c>
@@ -10972,7 +10967,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="341" spans="1:5">
+    <row r="341" customHeight="1" spans="1:5">
       <c r="A341" s="1" t="s">
         <v>1342</v>
       </c>
@@ -10989,7 +10984,7 @@
         <v>1344</v>
       </c>
     </row>
-    <row r="342" spans="1:5">
+    <row r="342" customHeight="1" spans="1:5">
       <c r="A342" s="1" t="s">
         <v>1345</v>
       </c>
@@ -11006,7 +11001,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="343" spans="1:5">
+    <row r="343" customHeight="1" spans="1:5">
       <c r="A343" s="1" t="s">
         <v>1348</v>
       </c>
@@ -11023,7 +11018,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="344" spans="1:5">
+    <row r="344" customHeight="1" spans="1:5">
       <c r="A344" s="1" t="s">
         <v>1351</v>
       </c>
@@ -11040,7 +11035,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="345" spans="1:5">
+    <row r="345" customHeight="1" spans="1:5">
       <c r="A345" s="1" t="s">
         <v>1354</v>
       </c>
@@ -11057,7 +11052,7 @@
         <v>1356</v>
       </c>
     </row>
-    <row r="346" spans="1:5">
+    <row r="346" customHeight="1" spans="1:5">
       <c r="A346" s="1" t="s">
         <v>1357</v>
       </c>
@@ -11074,7 +11069,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="347" spans="1:5">
+    <row r="347" customHeight="1" spans="1:5">
       <c r="A347" s="1" t="s">
         <v>1360</v>
       </c>
@@ -11091,7 +11086,7 @@
         <v>1362</v>
       </c>
     </row>
-    <row r="348" spans="1:5">
+    <row r="348" customHeight="1" spans="1:5">
       <c r="A348" s="1" t="s">
         <v>1363</v>
       </c>
@@ -11108,7 +11103,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="349" spans="1:5">
+    <row r="349" customHeight="1" spans="1:5">
       <c r="A349" s="1" t="s">
         <v>1366</v>
       </c>
@@ -11125,7 +11120,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="350" spans="1:5">
+    <row r="350" customHeight="1" spans="1:5">
       <c r="A350" s="1" t="s">
         <v>1369</v>
       </c>
@@ -11142,7 +11137,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="351" spans="1:5">
+    <row r="351" customHeight="1" spans="1:5">
       <c r="A351" s="1" t="s">
         <v>1372</v>
       </c>
@@ -11159,7 +11154,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="352" spans="1:5">
+    <row r="352" customHeight="1" spans="1:5">
       <c r="A352" s="1" t="s">
         <v>1375</v>
       </c>

</xml_diff>